<commit_message>
feat: adicionar colunas Imagem e Preco em todas as planilhas automaticamente
</commit_message>
<xml_diff>
--- a/amazon.xlsx
+++ b/amazon.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -426,6 +426,12 @@
       <c r="F1" t="str">
         <v>Badge</v>
       </c>
+      <c r="G1" t="str">
+        <v>Imagem</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Preco</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -446,10 +452,16 @@
       <c r="F2" t="str">
         <v>Prime</v>
       </c>
+      <c r="G2" t="str">
+        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/4/4a/Amazon_icon.svg/256px-Amazon_icon.svg.png</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Ver Oferta</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Amazon products with affiliate links and images
</commit_message>
<xml_diff>
--- a/amazon.xlsx
+++ b/amazon.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Links" sheetId="1" r:id="rId1"/>
+    <sheet name="Produtos" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,15 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="50.83203125" customWidth="1"/>
-    <col min="3" max="3" width="40.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,50 +410,78 @@
         <v>Link</v>
       </c>
       <c r="D1" t="str">
-        <v>Icone</v>
+        <v>Badge</v>
       </c>
       <c r="E1" t="str">
-        <v>CorIcone</v>
+        <v>Imagem</v>
       </c>
       <c r="F1" t="str">
-        <v>Badge</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Imagem</v>
-      </c>
-      <c r="H1" t="str">
         <v>Preco</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Echo Dot 5ª Geração</v>
+        <v>Echo Pop | Smart speaker compacto com Alexa</v>
       </c>
       <c r="B2" t="str">
-        <v>Smart Speaker com Alexa. O melhor som já feito.</v>
+        <v>O som que preenche o seu espaço com a Alexa integrada.</v>
       </c>
       <c r="C2" t="str">
-        <v>https://amazon.com.br</v>
+        <v>https://www.amazon.com.br/Echo-Pop-Cor-Preta/dp/B09WXVH7WK?tag=afiliadosbrab-20</v>
       </c>
       <c r="D2" t="str">
-        <v>speaker</v>
+        <v>Amazon</v>
       </c>
       <c r="E2" t="str">
-        <v>#ff9900</v>
+        <v>https://m.media-amazon.com/images/I/61vP1V9q7pL._AC_SL1000_.jpg</v>
       </c>
       <c r="F2" t="str">
-        <v>Prime</v>
-      </c>
-      <c r="G2" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/thumb/4/4a/Amazon_icon.svg/256px-Amazon_icon.svg.png</v>
-      </c>
-      <c r="H2" t="str">
+        <v>R$ 349,00</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Apple iPhone 16e de 128 GB — Branco</v>
+      </c>
+      <c r="B3" t="str">
+        <v>O novo iPhone 16e com design elegante e performance incrível.</v>
+      </c>
+      <c r="C3" t="str">
+        <v>https://amzn.to/48wdwEP</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Amazon</v>
+      </c>
+      <c r="E3" t="str">
+        <v>https://m.media-amazon.com/images/I/61v-DOWY16L._AC_SL1500_.jpg</v>
+      </c>
+      <c r="F3" t="str">
+        <v>R$ 3.699,00</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Echo Dot (5ª Geração)</v>
+      </c>
+      <c r="B4" t="str">
+        <v>O smart speaker com Alexa de melhor som já feito.</v>
+      </c>
+      <c r="C4" t="str">
+        <v>https://www.amazon.com.br/Echo-Dot-5%C2%AA-gera%C3%A7%C3%A3o-Preto/dp/B09B8VGMSY?tag=afiliadosbrab-20</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Amazon</v>
+      </c>
+      <c r="E4" t="str">
+        <v>https://m.media-amazon.com/images/I/61M63L99mYL._AC_SL1500_.jpg</v>
+      </c>
+      <c r="F4" t="str">
         <v>Ver Oferta</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Amazon products with local images and affiliate links
</commit_message>
<xml_diff>
--- a/amazon.xlsx
+++ b/amazon.xlsx
@@ -433,7 +433,7 @@
         <v>Amazon</v>
       </c>
       <c r="E2" t="str">
-        <v>https://m.media-amazon.com/images/I/61vP1V9q7pL._AC_SL1000_.jpg</v>
+        <v>assets/produtos/echo_pop.png</v>
       </c>
       <c r="F2" t="str">
         <v>R$ 349,00</v>
@@ -453,7 +453,7 @@
         <v>Amazon</v>
       </c>
       <c r="E3" t="str">
-        <v>https://m.media-amazon.com/images/I/61v-DOWY16L._AC_SL1500_.jpg</v>
+        <v>assets/produtos/iphone.png</v>
       </c>
       <c r="F3" t="str">
         <v>R$ 3.699,00</v>
@@ -473,7 +473,7 @@
         <v>Amazon</v>
       </c>
       <c r="E4" t="str">
-        <v>https://m.media-amazon.com/images/I/61M63L99mYL._AC_SL1500_.jpg</v>
+        <v>assets/produtos/echo_pop.png</v>
       </c>
       <c r="F4" t="str">
         <v>Ver Oferta</v>

</xml_diff>